<commit_message>
release: v2.2.0 (2026-08-23) - Fix Excel column alignments, EQUIPMENT_Data mappings, and indoor unit power rules
</commit_message>
<xml_diff>
--- a/backend/product_database/選機表-.xlsx
+++ b/backend/product_database/選機表-.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flitt\.gemini\antigravity\scratch\ac-selection-system\backend\product_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910B2A8E-75F0-4690-A5CD-849AC3410FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F9C188-4843-4B26-B789-9B5666ABBC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B12BA144-AC3D-4CE9-9615-9201C80CE143}"/>
+    <workbookView xWindow="1128" yWindow="300" windowWidth="11520" windowHeight="12240" xr2:uid="{B12BA144-AC3D-4CE9-9615-9201C80CE143}"/>
   </bookViews>
   <sheets>
     <sheet name="選機" sheetId="12" r:id="rId1"/>
@@ -3900,7 +3900,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -4272,9 +4272,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="188" fontId="3" fillId="11" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="3" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="3" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19654,7 +19651,7 @@
     <col min="29" max="30" width="10.6640625" style="16" customWidth="1"/>
     <col min="31" max="31" width="18.6640625" style="15" customWidth="1"/>
     <col min="32" max="32" width="5.6640625" style="15" customWidth="1"/>
-    <col min="33" max="33" width="10.44140625" style="14" hidden="1" customWidth="1"/>
+    <col min="33" max="33" width="10.44140625" style="14" customWidth="1"/>
     <col min="34" max="34" width="15.6640625" style="14" customWidth="1"/>
     <col min="35" max="35" width="7.21875" style="14" customWidth="1"/>
     <col min="36" max="36" width="7.33203125" style="18" customWidth="1"/>
@@ -19976,15 +19973,15 @@
       <c r="BF5" s="19"/>
     </row>
     <row r="6" spans="1:58" s="2" customFormat="1" ht="21" customHeight="1">
-      <c r="A6" s="129" t="s">
+      <c r="A6" s="128" t="s">
         <v>736</v>
       </c>
-      <c r="B6" s="130"/>
-      <c r="C6" s="130"/>
-      <c r="D6" s="130"/>
-      <c r="E6" s="130"/>
-      <c r="F6" s="130"/>
-      <c r="G6" s="130"/>
+      <c r="B6" s="129"/>
+      <c r="C6" s="129"/>
+      <c r="D6" s="129"/>
+      <c r="E6" s="129"/>
+      <c r="F6" s="129"/>
+      <c r="G6" s="129"/>
       <c r="H6" s="60"/>
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
@@ -20038,16 +20035,16 @@
       <c r="BF6" s="10"/>
     </row>
     <row r="7" spans="1:58" ht="39.75" customHeight="1">
-      <c r="A7" s="131" t="s">
+      <c r="A7" s="130" t="s">
         <v>691</v>
       </c>
-      <c r="B7" s="133" t="s">
+      <c r="B7" s="132" t="s">
         <v>692</v>
       </c>
-      <c r="C7" s="135" t="s">
+      <c r="C7" s="134" t="s">
         <v>693</v>
       </c>
-      <c r="D7" s="132" t="s">
+      <c r="D7" s="131" t="s">
         <v>694</v>
       </c>
       <c r="E7" s="64" t="s">
@@ -20059,87 +20056,87 @@
       <c r="G7" s="65" t="s">
         <v>697</v>
       </c>
-      <c r="H7" s="155" t="s">
+      <c r="H7" s="154" t="s">
         <v>738</v>
       </c>
-      <c r="I7" s="156"/>
-      <c r="J7" s="156"/>
-      <c r="K7" s="156"/>
-      <c r="L7" s="148" t="s">
+      <c r="I7" s="155"/>
+      <c r="J7" s="155"/>
+      <c r="K7" s="155"/>
+      <c r="L7" s="147" t="s">
         <v>698</v>
       </c>
-      <c r="M7" s="148"/>
-      <c r="N7" s="149" t="s">
+      <c r="M7" s="147"/>
+      <c r="N7" s="148" t="s">
         <v>699</v>
       </c>
-      <c r="O7" s="150"/>
-      <c r="P7" s="150"/>
-      <c r="Q7" s="150"/>
-      <c r="R7" s="150"/>
-      <c r="S7" s="150"/>
-      <c r="T7" s="150"/>
-      <c r="U7" s="150"/>
-      <c r="V7" s="151"/>
-      <c r="W7" s="152" t="s">
+      <c r="O7" s="149"/>
+      <c r="P7" s="149"/>
+      <c r="Q7" s="149"/>
+      <c r="R7" s="149"/>
+      <c r="S7" s="149"/>
+      <c r="T7" s="149"/>
+      <c r="U7" s="149"/>
+      <c r="V7" s="150"/>
+      <c r="W7" s="151" t="s">
         <v>700</v>
       </c>
-      <c r="X7" s="151"/>
-      <c r="Y7" s="153" t="s">
+      <c r="X7" s="150"/>
+      <c r="Y7" s="152" t="s">
         <v>701</v>
       </c>
       <c r="Z7" s="66" t="s">
         <v>702</v>
       </c>
-      <c r="AA7" s="152" t="s">
+      <c r="AA7" s="151" t="s">
         <v>703</v>
       </c>
-      <c r="AB7" s="150"/>
-      <c r="AC7" s="150"/>
-      <c r="AD7" s="151"/>
-      <c r="AE7" s="142" t="s">
+      <c r="AB7" s="149"/>
+      <c r="AC7" s="149"/>
+      <c r="AD7" s="150"/>
+      <c r="AE7" s="141" t="s">
         <v>704</v>
       </c>
-      <c r="AF7" s="142"/>
-      <c r="AG7" s="132"/>
-      <c r="AH7" s="132"/>
-      <c r="AI7" s="132"/>
-      <c r="AJ7" s="132"/>
-      <c r="AK7" s="132"/>
-      <c r="AL7" s="132"/>
-      <c r="AM7" s="132"/>
-      <c r="AN7" s="132"/>
-      <c r="AO7" s="132"/>
-      <c r="AP7" s="146" t="s">
+      <c r="AF7" s="141"/>
+      <c r="AG7" s="131"/>
+      <c r="AH7" s="131"/>
+      <c r="AI7" s="131"/>
+      <c r="AJ7" s="131"/>
+      <c r="AK7" s="131"/>
+      <c r="AL7" s="131"/>
+      <c r="AM7" s="131"/>
+      <c r="AN7" s="131"/>
+      <c r="AO7" s="131"/>
+      <c r="AP7" s="145" t="s">
         <v>2</v>
       </c>
-      <c r="AQ7" s="136" t="s">
+      <c r="AQ7" s="135" t="s">
         <v>14</v>
       </c>
-      <c r="AR7" s="137"/>
-      <c r="AS7" s="137"/>
-      <c r="AT7" s="137"/>
-      <c r="AU7" s="137"/>
-      <c r="AV7" s="137"/>
-      <c r="AW7" s="137"/>
-      <c r="AX7" s="137"/>
-      <c r="AY7" s="137"/>
-      <c r="AZ7" s="138"/>
-      <c r="BA7" s="139" t="s">
+      <c r="AR7" s="136"/>
+      <c r="AS7" s="136"/>
+      <c r="AT7" s="136"/>
+      <c r="AU7" s="136"/>
+      <c r="AV7" s="136"/>
+      <c r="AW7" s="136"/>
+      <c r="AX7" s="136"/>
+      <c r="AY7" s="136"/>
+      <c r="AZ7" s="137"/>
+      <c r="BA7" s="138" t="s">
         <v>705</v>
       </c>
-      <c r="BB7" s="140"/>
-      <c r="BC7" s="140"/>
-      <c r="BD7" s="141"/>
-      <c r="BE7" s="139" t="s">
+      <c r="BB7" s="139"/>
+      <c r="BC7" s="139"/>
+      <c r="BD7" s="140"/>
+      <c r="BE7" s="138" t="s">
         <v>706</v>
       </c>
-      <c r="BF7" s="141"/>
+      <c r="BF7" s="140"/>
     </row>
     <row r="8" spans="1:58" ht="51.75" customHeight="1">
-      <c r="A8" s="132"/>
-      <c r="B8" s="134"/>
-      <c r="C8" s="134"/>
-      <c r="D8" s="132"/>
+      <c r="A8" s="131"/>
+      <c r="B8" s="133"/>
+      <c r="C8" s="133"/>
+      <c r="D8" s="131"/>
       <c r="E8" s="64" t="s">
         <v>707</v>
       </c>
@@ -20200,7 +20197,7 @@
       <c r="X8" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="Y8" s="154"/>
+      <c r="Y8" s="153"/>
       <c r="Z8" s="73" t="s">
         <v>9</v>
       </c>
@@ -20249,7 +20246,7 @@
       <c r="AO8" s="76" t="s">
         <v>718</v>
       </c>
-      <c r="AP8" s="147"/>
+      <c r="AP8" s="146"/>
       <c r="AQ8" s="79" t="s">
         <v>727</v>
       </c>
@@ -20324,7 +20321,10 @@
       <c r="V9" s="100"/>
       <c r="W9" s="99"/>
       <c r="X9" s="88"/>
-      <c r="Y9" s="53"/>
+      <c r="Y9" s="53">
+        <f>R9*O9</f>
+        <v>0</v>
+      </c>
       <c r="Z9" s="53"/>
       <c r="AA9" s="104"/>
       <c r="AB9" s="105"/>
@@ -20332,7 +20332,10 @@
       <c r="AD9" s="106"/>
       <c r="AE9" s="107"/>
       <c r="AF9" s="108"/>
-      <c r="AG9" s="109"/>
+      <c r="AG9" s="109">
+        <f>AH9*860</f>
+        <v>0</v>
+      </c>
       <c r="AH9" s="110"/>
       <c r="AI9" s="102"/>
       <c r="AJ9" s="111"/>
@@ -20384,7 +20387,10 @@
       <c r="V10" s="122"/>
       <c r="W10" s="121"/>
       <c r="X10" s="88"/>
-      <c r="Y10" s="53"/>
+      <c r="Y10" s="53">
+        <f t="shared" ref="Y10:Y57" si="0">R10*O10</f>
+        <v>0</v>
+      </c>
       <c r="Z10" s="53"/>
       <c r="AA10" s="104"/>
       <c r="AB10" s="105"/>
@@ -20392,7 +20398,10 @@
       <c r="AD10" s="106"/>
       <c r="AE10" s="123"/>
       <c r="AF10" s="108"/>
-      <c r="AG10" s="124"/>
+      <c r="AG10" s="124">
+        <f t="shared" ref="AG10:AG57" si="1">AH10*860</f>
+        <v>0</v>
+      </c>
       <c r="AH10" s="125"/>
       <c r="AI10" s="102"/>
       <c r="AJ10" s="111"/>
@@ -20444,7 +20453,10 @@
       <c r="V11" s="122"/>
       <c r="W11" s="121"/>
       <c r="X11" s="88"/>
-      <c r="Y11" s="53"/>
+      <c r="Y11" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z11" s="53"/>
       <c r="AA11" s="104"/>
       <c r="AB11" s="105"/>
@@ -20452,7 +20464,10 @@
       <c r="AD11" s="106"/>
       <c r="AE11" s="123"/>
       <c r="AF11" s="108"/>
-      <c r="AG11" s="124"/>
+      <c r="AG11" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH11" s="125"/>
       <c r="AI11" s="102"/>
       <c r="AJ11" s="111"/>
@@ -20504,7 +20519,10 @@
       <c r="V12" s="122"/>
       <c r="W12" s="121"/>
       <c r="X12" s="88"/>
-      <c r="Y12" s="53"/>
+      <c r="Y12" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z12" s="53"/>
       <c r="AA12" s="104"/>
       <c r="AB12" s="105"/>
@@ -20512,7 +20530,10 @@
       <c r="AD12" s="106"/>
       <c r="AE12" s="123"/>
       <c r="AF12" s="108"/>
-      <c r="AG12" s="124"/>
+      <c r="AG12" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH12" s="125"/>
       <c r="AI12" s="102"/>
       <c r="AJ12" s="111"/>
@@ -20564,7 +20585,10 @@
       <c r="V13" s="122"/>
       <c r="W13" s="121"/>
       <c r="X13" s="88"/>
-      <c r="Y13" s="53"/>
+      <c r="Y13" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z13" s="53"/>
       <c r="AA13" s="104"/>
       <c r="AB13" s="105"/>
@@ -20572,7 +20596,10 @@
       <c r="AD13" s="106"/>
       <c r="AE13" s="123"/>
       <c r="AF13" s="108"/>
-      <c r="AG13" s="124"/>
+      <c r="AG13" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH13" s="125"/>
       <c r="AI13" s="102"/>
       <c r="AJ13" s="111"/>
@@ -20624,7 +20651,10 @@
       <c r="V14" s="122"/>
       <c r="W14" s="121"/>
       <c r="X14" s="88"/>
-      <c r="Y14" s="53"/>
+      <c r="Y14" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z14" s="53"/>
       <c r="AA14" s="104"/>
       <c r="AB14" s="105"/>
@@ -20632,7 +20662,10 @@
       <c r="AD14" s="106"/>
       <c r="AE14" s="123"/>
       <c r="AF14" s="108"/>
-      <c r="AG14" s="124"/>
+      <c r="AG14" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH14" s="125"/>
       <c r="AI14" s="102"/>
       <c r="AJ14" s="111"/>
@@ -20684,7 +20717,10 @@
       <c r="V15" s="122"/>
       <c r="W15" s="121"/>
       <c r="X15" s="88"/>
-      <c r="Y15" s="53"/>
+      <c r="Y15" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z15" s="53"/>
       <c r="AA15" s="104"/>
       <c r="AB15" s="105"/>
@@ -20692,7 +20728,10 @@
       <c r="AD15" s="106"/>
       <c r="AE15" s="123"/>
       <c r="AF15" s="108"/>
-      <c r="AG15" s="124"/>
+      <c r="AG15" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH15" s="125"/>
       <c r="AI15" s="102"/>
       <c r="AJ15" s="111"/>
@@ -20744,7 +20783,10 @@
       <c r="V16" s="122"/>
       <c r="W16" s="121"/>
       <c r="X16" s="88"/>
-      <c r="Y16" s="53"/>
+      <c r="Y16" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z16" s="53"/>
       <c r="AA16" s="104"/>
       <c r="AB16" s="105"/>
@@ -20752,7 +20794,10 @@
       <c r="AD16" s="106"/>
       <c r="AE16" s="123"/>
       <c r="AF16" s="108"/>
-      <c r="AG16" s="124"/>
+      <c r="AG16" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH16" s="125"/>
       <c r="AI16" s="102"/>
       <c r="AJ16" s="111"/>
@@ -20804,7 +20849,10 @@
       <c r="V17" s="122"/>
       <c r="W17" s="121"/>
       <c r="X17" s="88"/>
-      <c r="Y17" s="53"/>
+      <c r="Y17" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z17" s="53"/>
       <c r="AA17" s="104"/>
       <c r="AB17" s="105"/>
@@ -20812,7 +20860,10 @@
       <c r="AD17" s="106"/>
       <c r="AE17" s="123"/>
       <c r="AF17" s="108"/>
-      <c r="AG17" s="124"/>
+      <c r="AG17" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH17" s="125"/>
       <c r="AI17" s="102"/>
       <c r="AJ17" s="111"/>
@@ -20864,7 +20915,10 @@
       <c r="V18" s="122"/>
       <c r="W18" s="121"/>
       <c r="X18" s="88"/>
-      <c r="Y18" s="53"/>
+      <c r="Y18" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z18" s="53"/>
       <c r="AA18" s="104"/>
       <c r="AB18" s="105"/>
@@ -20872,8 +20926,11 @@
       <c r="AD18" s="106"/>
       <c r="AE18" s="126"/>
       <c r="AF18" s="118"/>
-      <c r="AG18" s="127"/>
-      <c r="AH18" s="128"/>
+      <c r="AG18" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH18" s="127"/>
       <c r="AI18" s="102"/>
       <c r="AJ18" s="111"/>
       <c r="AK18" s="112"/>
@@ -20924,7 +20981,10 @@
       <c r="V19" s="122"/>
       <c r="W19" s="121"/>
       <c r="X19" s="88"/>
-      <c r="Y19" s="53"/>
+      <c r="Y19" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z19" s="53"/>
       <c r="AA19" s="104"/>
       <c r="AB19" s="105"/>
@@ -20932,8 +20992,11 @@
       <c r="AD19" s="106"/>
       <c r="AE19" s="126"/>
       <c r="AF19" s="118"/>
-      <c r="AG19" s="127"/>
-      <c r="AH19" s="128"/>
+      <c r="AG19" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH19" s="127"/>
       <c r="AI19" s="102"/>
       <c r="AJ19" s="111"/>
       <c r="AK19" s="112"/>
@@ -20984,7 +21047,10 @@
       <c r="V20" s="122"/>
       <c r="W20" s="121"/>
       <c r="X20" s="88"/>
-      <c r="Y20" s="53"/>
+      <c r="Y20" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z20" s="53"/>
       <c r="AA20" s="104"/>
       <c r="AB20" s="105"/>
@@ -20992,8 +21058,11 @@
       <c r="AD20" s="106"/>
       <c r="AE20" s="126"/>
       <c r="AF20" s="118"/>
-      <c r="AG20" s="127"/>
-      <c r="AH20" s="128"/>
+      <c r="AG20" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH20" s="127"/>
       <c r="AI20" s="102"/>
       <c r="AJ20" s="111"/>
       <c r="AK20" s="112"/>
@@ -21044,7 +21113,10 @@
       <c r="V21" s="122"/>
       <c r="W21" s="121"/>
       <c r="X21" s="88"/>
-      <c r="Y21" s="53"/>
+      <c r="Y21" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z21" s="53"/>
       <c r="AA21" s="104"/>
       <c r="AB21" s="105"/>
@@ -21052,8 +21124,11 @@
       <c r="AD21" s="106"/>
       <c r="AE21" s="126"/>
       <c r="AF21" s="118"/>
-      <c r="AG21" s="127"/>
-      <c r="AH21" s="128"/>
+      <c r="AG21" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH21" s="127"/>
       <c r="AI21" s="102"/>
       <c r="AJ21" s="111"/>
       <c r="AK21" s="112"/>
@@ -21104,7 +21179,10 @@
       <c r="V22" s="122"/>
       <c r="W22" s="121"/>
       <c r="X22" s="88"/>
-      <c r="Y22" s="53"/>
+      <c r="Y22" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z22" s="53"/>
       <c r="AA22" s="104"/>
       <c r="AB22" s="105"/>
@@ -21112,7 +21190,10 @@
       <c r="AD22" s="106"/>
       <c r="AE22" s="123"/>
       <c r="AF22" s="108"/>
-      <c r="AG22" s="124"/>
+      <c r="AG22" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH22" s="125"/>
       <c r="AI22" s="102"/>
       <c r="AJ22" s="111"/>
@@ -21164,7 +21245,10 @@
       <c r="V23" s="122"/>
       <c r="W23" s="121"/>
       <c r="X23" s="88"/>
-      <c r="Y23" s="53"/>
+      <c r="Y23" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z23" s="53"/>
       <c r="AA23" s="104"/>
       <c r="AB23" s="105"/>
@@ -21172,7 +21256,10 @@
       <c r="AD23" s="106"/>
       <c r="AE23" s="123"/>
       <c r="AF23" s="108"/>
-      <c r="AG23" s="124"/>
+      <c r="AG23" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH23" s="125"/>
       <c r="AI23" s="102"/>
       <c r="AJ23" s="111"/>
@@ -21224,7 +21311,10 @@
       <c r="V24" s="122"/>
       <c r="W24" s="121"/>
       <c r="X24" s="88"/>
-      <c r="Y24" s="53"/>
+      <c r="Y24" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z24" s="53"/>
       <c r="AA24" s="104"/>
       <c r="AB24" s="105"/>
@@ -21232,7 +21322,10 @@
       <c r="AD24" s="106"/>
       <c r="AE24" s="123"/>
       <c r="AF24" s="108"/>
-      <c r="AG24" s="124"/>
+      <c r="AG24" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH24" s="125"/>
       <c r="AI24" s="102"/>
       <c r="AJ24" s="111"/>
@@ -21284,7 +21377,10 @@
       <c r="V25" s="122"/>
       <c r="W25" s="121"/>
       <c r="X25" s="88"/>
-      <c r="Y25" s="53"/>
+      <c r="Y25" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z25" s="53"/>
       <c r="AA25" s="104"/>
       <c r="AB25" s="105"/>
@@ -21292,7 +21388,10 @@
       <c r="AD25" s="106"/>
       <c r="AE25" s="123"/>
       <c r="AF25" s="108"/>
-      <c r="AG25" s="124"/>
+      <c r="AG25" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH25" s="125"/>
       <c r="AI25" s="102"/>
       <c r="AJ25" s="111"/>
@@ -21344,7 +21443,10 @@
       <c r="V26" s="122"/>
       <c r="W26" s="121"/>
       <c r="X26" s="88"/>
-      <c r="Y26" s="53"/>
+      <c r="Y26" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z26" s="53"/>
       <c r="AA26" s="104"/>
       <c r="AB26" s="105"/>
@@ -21352,7 +21454,10 @@
       <c r="AD26" s="106"/>
       <c r="AE26" s="123"/>
       <c r="AF26" s="108"/>
-      <c r="AG26" s="124"/>
+      <c r="AG26" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH26" s="125"/>
       <c r="AI26" s="102"/>
       <c r="AJ26" s="111"/>
@@ -21404,7 +21509,10 @@
       <c r="V27" s="122"/>
       <c r="W27" s="121"/>
       <c r="X27" s="88"/>
-      <c r="Y27" s="53"/>
+      <c r="Y27" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z27" s="53"/>
       <c r="AA27" s="104"/>
       <c r="AB27" s="105"/>
@@ -21412,7 +21520,10 @@
       <c r="AD27" s="106"/>
       <c r="AE27" s="123"/>
       <c r="AF27" s="108"/>
-      <c r="AG27" s="124"/>
+      <c r="AG27" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH27" s="125"/>
       <c r="AI27" s="102"/>
       <c r="AJ27" s="111"/>
@@ -21464,7 +21575,10 @@
       <c r="V28" s="122"/>
       <c r="W28" s="121"/>
       <c r="X28" s="88"/>
-      <c r="Y28" s="53"/>
+      <c r="Y28" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z28" s="53"/>
       <c r="AA28" s="104"/>
       <c r="AB28" s="105"/>
@@ -21472,7 +21586,10 @@
       <c r="AD28" s="106"/>
       <c r="AE28" s="123"/>
       <c r="AF28" s="108"/>
-      <c r="AG28" s="124"/>
+      <c r="AG28" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH28" s="125"/>
       <c r="AI28" s="102"/>
       <c r="AJ28" s="111"/>
@@ -21524,7 +21641,10 @@
       <c r="V29" s="122"/>
       <c r="W29" s="121"/>
       <c r="X29" s="88"/>
-      <c r="Y29" s="53"/>
+      <c r="Y29" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z29" s="53"/>
       <c r="AA29" s="104"/>
       <c r="AB29" s="105"/>
@@ -21532,7 +21652,10 @@
       <c r="AD29" s="106"/>
       <c r="AE29" s="123"/>
       <c r="AF29" s="108"/>
-      <c r="AG29" s="124"/>
+      <c r="AG29" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH29" s="125"/>
       <c r="AI29" s="102"/>
       <c r="AJ29" s="111"/>
@@ -21584,7 +21707,10 @@
       <c r="V30" s="122"/>
       <c r="W30" s="121"/>
       <c r="X30" s="88"/>
-      <c r="Y30" s="53"/>
+      <c r="Y30" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z30" s="53"/>
       <c r="AA30" s="104"/>
       <c r="AB30" s="105"/>
@@ -21592,8 +21718,11 @@
       <c r="AD30" s="106"/>
       <c r="AE30" s="126"/>
       <c r="AF30" s="118"/>
-      <c r="AG30" s="127"/>
-      <c r="AH30" s="128"/>
+      <c r="AG30" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH30" s="127"/>
       <c r="AI30" s="102"/>
       <c r="AJ30" s="111"/>
       <c r="AK30" s="112"/>
@@ -21644,7 +21773,10 @@
       <c r="V31" s="122"/>
       <c r="W31" s="121"/>
       <c r="X31" s="88"/>
-      <c r="Y31" s="53"/>
+      <c r="Y31" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z31" s="53"/>
       <c r="AA31" s="104"/>
       <c r="AB31" s="105"/>
@@ -21652,8 +21784,11 @@
       <c r="AD31" s="106"/>
       <c r="AE31" s="126"/>
       <c r="AF31" s="118"/>
-      <c r="AG31" s="127"/>
-      <c r="AH31" s="128"/>
+      <c r="AG31" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH31" s="127"/>
       <c r="AI31" s="102"/>
       <c r="AJ31" s="111"/>
       <c r="AK31" s="112"/>
@@ -21704,7 +21839,10 @@
       <c r="V32" s="122"/>
       <c r="W32" s="121"/>
       <c r="X32" s="88"/>
-      <c r="Y32" s="53"/>
+      <c r="Y32" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z32" s="53"/>
       <c r="AA32" s="104"/>
       <c r="AB32" s="105"/>
@@ -21712,8 +21850,11 @@
       <c r="AD32" s="106"/>
       <c r="AE32" s="126"/>
       <c r="AF32" s="118"/>
-      <c r="AG32" s="127"/>
-      <c r="AH32" s="128"/>
+      <c r="AG32" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH32" s="127"/>
       <c r="AI32" s="102"/>
       <c r="AJ32" s="111"/>
       <c r="AK32" s="112"/>
@@ -21764,7 +21905,10 @@
       <c r="V33" s="122"/>
       <c r="W33" s="121"/>
       <c r="X33" s="88"/>
-      <c r="Y33" s="53"/>
+      <c r="Y33" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z33" s="53"/>
       <c r="AA33" s="104"/>
       <c r="AB33" s="105"/>
@@ -21772,8 +21916,11 @@
       <c r="AD33" s="106"/>
       <c r="AE33" s="126"/>
       <c r="AF33" s="118"/>
-      <c r="AG33" s="127"/>
-      <c r="AH33" s="128"/>
+      <c r="AG33" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH33" s="127"/>
       <c r="AI33" s="102"/>
       <c r="AJ33" s="111"/>
       <c r="AK33" s="112"/>
@@ -21824,7 +21971,10 @@
       <c r="V34" s="122"/>
       <c r="W34" s="121"/>
       <c r="X34" s="88"/>
-      <c r="Y34" s="53"/>
+      <c r="Y34" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z34" s="53"/>
       <c r="AA34" s="104"/>
       <c r="AB34" s="105"/>
@@ -21832,7 +21982,10 @@
       <c r="AD34" s="106"/>
       <c r="AE34" s="123"/>
       <c r="AF34" s="108"/>
-      <c r="AG34" s="124"/>
+      <c r="AG34" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH34" s="125"/>
       <c r="AI34" s="102"/>
       <c r="AJ34" s="111"/>
@@ -21884,7 +22037,10 @@
       <c r="V35" s="122"/>
       <c r="W35" s="121"/>
       <c r="X35" s="88"/>
-      <c r="Y35" s="53"/>
+      <c r="Y35" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z35" s="53"/>
       <c r="AA35" s="104"/>
       <c r="AB35" s="105"/>
@@ -21892,7 +22048,10 @@
       <c r="AD35" s="106"/>
       <c r="AE35" s="123"/>
       <c r="AF35" s="108"/>
-      <c r="AG35" s="124"/>
+      <c r="AG35" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH35" s="125"/>
       <c r="AI35" s="102"/>
       <c r="AJ35" s="111"/>
@@ -21944,7 +22103,10 @@
       <c r="V36" s="122"/>
       <c r="W36" s="121"/>
       <c r="X36" s="88"/>
-      <c r="Y36" s="53"/>
+      <c r="Y36" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z36" s="53"/>
       <c r="AA36" s="104"/>
       <c r="AB36" s="105"/>
@@ -21952,7 +22114,10 @@
       <c r="AD36" s="106"/>
       <c r="AE36" s="123"/>
       <c r="AF36" s="108"/>
-      <c r="AG36" s="124"/>
+      <c r="AG36" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH36" s="125"/>
       <c r="AI36" s="102"/>
       <c r="AJ36" s="111"/>
@@ -22004,7 +22169,10 @@
       <c r="V37" s="122"/>
       <c r="W37" s="121"/>
       <c r="X37" s="88"/>
-      <c r="Y37" s="53"/>
+      <c r="Y37" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z37" s="53"/>
       <c r="AA37" s="104"/>
       <c r="AB37" s="105"/>
@@ -22012,7 +22180,10 @@
       <c r="AD37" s="106"/>
       <c r="AE37" s="123"/>
       <c r="AF37" s="108"/>
-      <c r="AG37" s="124"/>
+      <c r="AG37" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH37" s="125"/>
       <c r="AI37" s="102"/>
       <c r="AJ37" s="111"/>
@@ -22064,7 +22235,10 @@
       <c r="V38" s="122"/>
       <c r="W38" s="121"/>
       <c r="X38" s="88"/>
-      <c r="Y38" s="53"/>
+      <c r="Y38" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z38" s="53"/>
       <c r="AA38" s="104"/>
       <c r="AB38" s="105"/>
@@ -22072,7 +22246,10 @@
       <c r="AD38" s="106"/>
       <c r="AE38" s="123"/>
       <c r="AF38" s="108"/>
-      <c r="AG38" s="124"/>
+      <c r="AG38" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH38" s="125"/>
       <c r="AI38" s="102"/>
       <c r="AJ38" s="111"/>
@@ -22124,7 +22301,10 @@
       <c r="V39" s="122"/>
       <c r="W39" s="121"/>
       <c r="X39" s="88"/>
-      <c r="Y39" s="53"/>
+      <c r="Y39" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z39" s="53"/>
       <c r="AA39" s="104"/>
       <c r="AB39" s="105"/>
@@ -22132,7 +22312,10 @@
       <c r="AD39" s="106"/>
       <c r="AE39" s="123"/>
       <c r="AF39" s="108"/>
-      <c r="AG39" s="124"/>
+      <c r="AG39" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH39" s="125"/>
       <c r="AI39" s="102"/>
       <c r="AJ39" s="111"/>
@@ -22184,7 +22367,10 @@
       <c r="V40" s="122"/>
       <c r="W40" s="121"/>
       <c r="X40" s="88"/>
-      <c r="Y40" s="53"/>
+      <c r="Y40" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z40" s="53"/>
       <c r="AA40" s="104"/>
       <c r="AB40" s="105"/>
@@ -22192,7 +22378,10 @@
       <c r="AD40" s="106"/>
       <c r="AE40" s="123"/>
       <c r="AF40" s="108"/>
-      <c r="AG40" s="124"/>
+      <c r="AG40" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH40" s="125"/>
       <c r="AI40" s="102"/>
       <c r="AJ40" s="111"/>
@@ -22244,7 +22433,10 @@
       <c r="V41" s="122"/>
       <c r="W41" s="121"/>
       <c r="X41" s="88"/>
-      <c r="Y41" s="53"/>
+      <c r="Y41" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z41" s="53"/>
       <c r="AA41" s="104"/>
       <c r="AB41" s="105"/>
@@ -22252,7 +22444,10 @@
       <c r="AD41" s="106"/>
       <c r="AE41" s="123"/>
       <c r="AF41" s="108"/>
-      <c r="AG41" s="124"/>
+      <c r="AG41" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH41" s="125"/>
       <c r="AI41" s="102"/>
       <c r="AJ41" s="111"/>
@@ -22304,7 +22499,10 @@
       <c r="V42" s="122"/>
       <c r="W42" s="121"/>
       <c r="X42" s="88"/>
-      <c r="Y42" s="53"/>
+      <c r="Y42" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z42" s="53"/>
       <c r="AA42" s="104"/>
       <c r="AB42" s="105"/>
@@ -22312,8 +22510,11 @@
       <c r="AD42" s="106"/>
       <c r="AE42" s="126"/>
       <c r="AF42" s="118"/>
-      <c r="AG42" s="127"/>
-      <c r="AH42" s="128"/>
+      <c r="AG42" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH42" s="127"/>
       <c r="AI42" s="102"/>
       <c r="AJ42" s="111"/>
       <c r="AK42" s="112"/>
@@ -22364,7 +22565,10 @@
       <c r="V43" s="122"/>
       <c r="W43" s="121"/>
       <c r="X43" s="88"/>
-      <c r="Y43" s="53"/>
+      <c r="Y43" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z43" s="53"/>
       <c r="AA43" s="104"/>
       <c r="AB43" s="105"/>
@@ -22372,8 +22576,11 @@
       <c r="AD43" s="106"/>
       <c r="AE43" s="126"/>
       <c r="AF43" s="118"/>
-      <c r="AG43" s="127"/>
-      <c r="AH43" s="128"/>
+      <c r="AG43" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH43" s="127"/>
       <c r="AI43" s="102"/>
       <c r="AJ43" s="111"/>
       <c r="AK43" s="112"/>
@@ -22424,7 +22631,10 @@
       <c r="V44" s="122"/>
       <c r="W44" s="121"/>
       <c r="X44" s="88"/>
-      <c r="Y44" s="53"/>
+      <c r="Y44" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z44" s="53"/>
       <c r="AA44" s="104"/>
       <c r="AB44" s="105"/>
@@ -22432,8 +22642,11 @@
       <c r="AD44" s="106"/>
       <c r="AE44" s="126"/>
       <c r="AF44" s="118"/>
-      <c r="AG44" s="127"/>
-      <c r="AH44" s="128"/>
+      <c r="AG44" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH44" s="127"/>
       <c r="AI44" s="102"/>
       <c r="AJ44" s="111"/>
       <c r="AK44" s="112"/>
@@ -22484,7 +22697,10 @@
       <c r="V45" s="122"/>
       <c r="W45" s="121"/>
       <c r="X45" s="88"/>
-      <c r="Y45" s="53"/>
+      <c r="Y45" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z45" s="53"/>
       <c r="AA45" s="104"/>
       <c r="AB45" s="105"/>
@@ -22492,8 +22708,11 @@
       <c r="AD45" s="106"/>
       <c r="AE45" s="126"/>
       <c r="AF45" s="118"/>
-      <c r="AG45" s="127"/>
-      <c r="AH45" s="128"/>
+      <c r="AG45" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH45" s="127"/>
       <c r="AI45" s="102"/>
       <c r="AJ45" s="111"/>
       <c r="AK45" s="112"/>
@@ -22544,7 +22763,10 @@
       <c r="V46" s="122"/>
       <c r="W46" s="121"/>
       <c r="X46" s="88"/>
-      <c r="Y46" s="53"/>
+      <c r="Y46" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z46" s="53"/>
       <c r="AA46" s="104"/>
       <c r="AB46" s="105"/>
@@ -22552,7 +22774,10 @@
       <c r="AD46" s="106"/>
       <c r="AE46" s="123"/>
       <c r="AF46" s="108"/>
-      <c r="AG46" s="124"/>
+      <c r="AG46" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH46" s="125"/>
       <c r="AI46" s="102"/>
       <c r="AJ46" s="111"/>
@@ -22604,7 +22829,10 @@
       <c r="V47" s="122"/>
       <c r="W47" s="121"/>
       <c r="X47" s="88"/>
-      <c r="Y47" s="53"/>
+      <c r="Y47" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z47" s="53"/>
       <c r="AA47" s="104"/>
       <c r="AB47" s="105"/>
@@ -22612,7 +22840,10 @@
       <c r="AD47" s="106"/>
       <c r="AE47" s="123"/>
       <c r="AF47" s="108"/>
-      <c r="AG47" s="124"/>
+      <c r="AG47" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH47" s="125"/>
       <c r="AI47" s="102"/>
       <c r="AJ47" s="111"/>
@@ -22664,7 +22895,10 @@
       <c r="V48" s="122"/>
       <c r="W48" s="121"/>
       <c r="X48" s="88"/>
-      <c r="Y48" s="53"/>
+      <c r="Y48" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z48" s="53"/>
       <c r="AA48" s="104"/>
       <c r="AB48" s="105"/>
@@ -22672,7 +22906,10 @@
       <c r="AD48" s="106"/>
       <c r="AE48" s="123"/>
       <c r="AF48" s="108"/>
-      <c r="AG48" s="124"/>
+      <c r="AG48" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH48" s="125"/>
       <c r="AI48" s="102"/>
       <c r="AJ48" s="111"/>
@@ -22724,7 +22961,10 @@
       <c r="V49" s="122"/>
       <c r="W49" s="121"/>
       <c r="X49" s="88"/>
-      <c r="Y49" s="53"/>
+      <c r="Y49" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z49" s="53"/>
       <c r="AA49" s="104"/>
       <c r="AB49" s="105"/>
@@ -22732,7 +22972,10 @@
       <c r="AD49" s="106"/>
       <c r="AE49" s="123"/>
       <c r="AF49" s="108"/>
-      <c r="AG49" s="124"/>
+      <c r="AG49" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH49" s="125"/>
       <c r="AI49" s="102"/>
       <c r="AJ49" s="111"/>
@@ -22784,7 +23027,10 @@
       <c r="V50" s="122"/>
       <c r="W50" s="121"/>
       <c r="X50" s="88"/>
-      <c r="Y50" s="53"/>
+      <c r="Y50" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z50" s="53"/>
       <c r="AA50" s="104"/>
       <c r="AB50" s="105"/>
@@ -22792,7 +23038,10 @@
       <c r="AD50" s="106"/>
       <c r="AE50" s="123"/>
       <c r="AF50" s="108"/>
-      <c r="AG50" s="124"/>
+      <c r="AG50" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH50" s="125"/>
       <c r="AI50" s="102"/>
       <c r="AJ50" s="111"/>
@@ -22844,7 +23093,10 @@
       <c r="V51" s="122"/>
       <c r="W51" s="121"/>
       <c r="X51" s="88"/>
-      <c r="Y51" s="53"/>
+      <c r="Y51" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z51" s="53"/>
       <c r="AA51" s="104"/>
       <c r="AB51" s="105"/>
@@ -22852,7 +23104,10 @@
       <c r="AD51" s="106"/>
       <c r="AE51" s="123"/>
       <c r="AF51" s="108"/>
-      <c r="AG51" s="124"/>
+      <c r="AG51" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH51" s="125"/>
       <c r="AI51" s="102"/>
       <c r="AJ51" s="111"/>
@@ -22904,7 +23159,10 @@
       <c r="V52" s="122"/>
       <c r="W52" s="121"/>
       <c r="X52" s="88"/>
-      <c r="Y52" s="53"/>
+      <c r="Y52" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z52" s="53"/>
       <c r="AA52" s="104"/>
       <c r="AB52" s="105"/>
@@ -22912,7 +23170,10 @@
       <c r="AD52" s="106"/>
       <c r="AE52" s="123"/>
       <c r="AF52" s="108"/>
-      <c r="AG52" s="124"/>
+      <c r="AG52" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH52" s="125"/>
       <c r="AI52" s="102"/>
       <c r="AJ52" s="111"/>
@@ -22964,7 +23225,10 @@
       <c r="V53" s="122"/>
       <c r="W53" s="121"/>
       <c r="X53" s="88"/>
-      <c r="Y53" s="53"/>
+      <c r="Y53" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z53" s="53"/>
       <c r="AA53" s="104"/>
       <c r="AB53" s="105"/>
@@ -22972,7 +23236,10 @@
       <c r="AD53" s="106"/>
       <c r="AE53" s="123"/>
       <c r="AF53" s="108"/>
-      <c r="AG53" s="124"/>
+      <c r="AG53" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="AH53" s="125"/>
       <c r="AI53" s="102"/>
       <c r="AJ53" s="111"/>
@@ -23024,7 +23291,10 @@
       <c r="V54" s="100"/>
       <c r="W54" s="99"/>
       <c r="X54" s="88"/>
-      <c r="Y54" s="53"/>
+      <c r="Y54" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z54" s="53"/>
       <c r="AA54" s="104"/>
       <c r="AB54" s="105"/>
@@ -23032,8 +23302,11 @@
       <c r="AD54" s="106"/>
       <c r="AE54" s="126"/>
       <c r="AF54" s="118"/>
-      <c r="AG54" s="127"/>
-      <c r="AH54" s="128"/>
+      <c r="AG54" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH54" s="127"/>
       <c r="AI54" s="102"/>
       <c r="AJ54" s="111"/>
       <c r="AK54" s="112"/>
@@ -23084,7 +23357,10 @@
       <c r="V55" s="100"/>
       <c r="W55" s="99"/>
       <c r="X55" s="88"/>
-      <c r="Y55" s="53"/>
+      <c r="Y55" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z55" s="53"/>
       <c r="AA55" s="104"/>
       <c r="AB55" s="105"/>
@@ -23092,8 +23368,11 @@
       <c r="AD55" s="106"/>
       <c r="AE55" s="126"/>
       <c r="AF55" s="118"/>
-      <c r="AG55" s="127"/>
-      <c r="AH55" s="128"/>
+      <c r="AG55" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH55" s="127"/>
       <c r="AI55" s="102"/>
       <c r="AJ55" s="111"/>
       <c r="AK55" s="112"/>
@@ -23144,7 +23423,10 @@
       <c r="V56" s="100"/>
       <c r="W56" s="99"/>
       <c r="X56" s="88"/>
-      <c r="Y56" s="53"/>
+      <c r="Y56" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z56" s="53"/>
       <c r="AA56" s="104"/>
       <c r="AB56" s="105"/>
@@ -23152,8 +23434,11 @@
       <c r="AD56" s="106"/>
       <c r="AE56" s="126"/>
       <c r="AF56" s="118"/>
-      <c r="AG56" s="127"/>
-      <c r="AH56" s="128"/>
+      <c r="AG56" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH56" s="127"/>
       <c r="AI56" s="102"/>
       <c r="AJ56" s="111"/>
       <c r="AK56" s="112"/>
@@ -23204,7 +23489,10 @@
       <c r="V57" s="100"/>
       <c r="W57" s="99"/>
       <c r="X57" s="88"/>
-      <c r="Y57" s="53"/>
+      <c r="Y57" s="53">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="Z57" s="53"/>
       <c r="AA57" s="104"/>
       <c r="AB57" s="105"/>
@@ -23212,8 +23500,11 @@
       <c r="AD57" s="106"/>
       <c r="AE57" s="126"/>
       <c r="AF57" s="118"/>
-      <c r="AG57" s="127"/>
-      <c r="AH57" s="128"/>
+      <c r="AG57" s="124">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH57" s="127"/>
       <c r="AI57" s="102"/>
       <c r="AJ57" s="111"/>
       <c r="AK57" s="112"/>
@@ -23240,48 +23531,48 @@
       <c r="BF57" s="114"/>
     </row>
     <row r="58" spans="1:58" ht="24.9" customHeight="1">
-      <c r="A58" s="143"/>
-      <c r="B58" s="144"/>
-      <c r="C58" s="144"/>
-      <c r="D58" s="144"/>
-      <c r="E58" s="144"/>
-      <c r="F58" s="144"/>
-      <c r="G58" s="144"/>
-      <c r="H58" s="144"/>
-      <c r="I58" s="144"/>
-      <c r="J58" s="144"/>
-      <c r="K58" s="144"/>
-      <c r="L58" s="144"/>
-      <c r="M58" s="144"/>
-      <c r="N58" s="144"/>
-      <c r="O58" s="144"/>
-      <c r="P58" s="144"/>
-      <c r="Q58" s="144"/>
-      <c r="R58" s="144"/>
-      <c r="S58" s="144"/>
-      <c r="T58" s="144"/>
-      <c r="U58" s="144"/>
-      <c r="V58" s="144"/>
-      <c r="W58" s="144"/>
-      <c r="X58" s="144"/>
-      <c r="Y58" s="144"/>
-      <c r="Z58" s="144"/>
-      <c r="AA58" s="144"/>
-      <c r="AB58" s="144"/>
-      <c r="AC58" s="144"/>
-      <c r="AD58" s="144"/>
-      <c r="AE58" s="144"/>
-      <c r="AF58" s="144"/>
-      <c r="AG58" s="144"/>
-      <c r="AH58" s="144"/>
-      <c r="AI58" s="144"/>
-      <c r="AJ58" s="144"/>
-      <c r="AK58" s="144"/>
-      <c r="AL58" s="144"/>
-      <c r="AM58" s="144"/>
-      <c r="AN58" s="144"/>
-      <c r="AO58" s="144"/>
-      <c r="AP58" s="145"/>
+      <c r="A58" s="142"/>
+      <c r="B58" s="143"/>
+      <c r="C58" s="143"/>
+      <c r="D58" s="143"/>
+      <c r="E58" s="143"/>
+      <c r="F58" s="143"/>
+      <c r="G58" s="143"/>
+      <c r="H58" s="143"/>
+      <c r="I58" s="143"/>
+      <c r="J58" s="143"/>
+      <c r="K58" s="143"/>
+      <c r="L58" s="143"/>
+      <c r="M58" s="143"/>
+      <c r="N58" s="143"/>
+      <c r="O58" s="143"/>
+      <c r="P58" s="143"/>
+      <c r="Q58" s="143"/>
+      <c r="R58" s="143"/>
+      <c r="S58" s="143"/>
+      <c r="T58" s="143"/>
+      <c r="U58" s="143"/>
+      <c r="V58" s="143"/>
+      <c r="W58" s="143"/>
+      <c r="X58" s="143"/>
+      <c r="Y58" s="143"/>
+      <c r="Z58" s="143"/>
+      <c r="AA58" s="143"/>
+      <c r="AB58" s="143"/>
+      <c r="AC58" s="143"/>
+      <c r="AD58" s="143"/>
+      <c r="AE58" s="143"/>
+      <c r="AF58" s="143"/>
+      <c r="AG58" s="143"/>
+      <c r="AH58" s="143"/>
+      <c r="AI58" s="143"/>
+      <c r="AJ58" s="143"/>
+      <c r="AK58" s="143"/>
+      <c r="AL58" s="143"/>
+      <c r="AM58" s="143"/>
+      <c r="AN58" s="143"/>
+      <c r="AO58" s="143"/>
+      <c r="AP58" s="144"/>
       <c r="AQ58" s="113"/>
       <c r="AR58" s="114">
         <v>2</v>
@@ -23290,7 +23581,7 @@
         <v>25</v>
       </c>
       <c r="AT58" s="88">
-        <f t="shared" ref="AT58" si="0">AR58*AS58</f>
+        <f t="shared" ref="AT58" si="2">AR58*AS58</f>
         <v>50</v>
       </c>
       <c r="AU58" s="114"/>
@@ -23538,34 +23829,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:27">
-      <c r="B2" s="157" t="s">
+      <c r="B2" s="156" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="158"/>
-      <c r="D2" s="158"/>
-      <c r="E2" s="158"/>
-      <c r="F2" s="158"/>
-      <c r="G2" s="158"/>
-      <c r="H2" s="158"/>
-      <c r="I2" s="158"/>
-      <c r="J2" s="158"/>
-      <c r="M2" s="159" t="s">
+      <c r="C2" s="157"/>
+      <c r="D2" s="157"/>
+      <c r="E2" s="157"/>
+      <c r="F2" s="157"/>
+      <c r="G2" s="157"/>
+      <c r="H2" s="157"/>
+      <c r="I2" s="157"/>
+      <c r="J2" s="157"/>
+      <c r="M2" s="158" t="s">
         <v>17</v>
       </c>
-      <c r="N2" s="159"/>
-      <c r="O2" s="159"/>
-      <c r="P2" s="159"/>
-      <c r="Q2" s="159"/>
-      <c r="R2" s="159"/>
+      <c r="N2" s="158"/>
+      <c r="O2" s="158"/>
+      <c r="P2" s="158"/>
+      <c r="Q2" s="158"/>
+      <c r="R2" s="158"/>
       <c r="S2" s="22"/>
       <c r="T2" s="22"/>
-      <c r="V2" s="160" t="s">
+      <c r="V2" s="159" t="s">
         <v>18</v>
       </c>
-      <c r="W2" s="160"/>
-      <c r="X2" s="160"/>
-      <c r="Y2" s="160"/>
-      <c r="Z2" s="160"/>
+      <c r="W2" s="159"/>
+      <c r="X2" s="159"/>
+      <c r="Y2" s="159"/>
+      <c r="Z2" s="159"/>
     </row>
     <row r="3" spans="2:27" ht="48.6">
       <c r="B3" s="23" t="s">
@@ -24427,12 +24718,12 @@
       <c r="T17" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="V17" s="160" t="s">
+      <c r="V17" s="159" t="s">
         <v>82</v>
       </c>
-      <c r="W17" s="160"/>
-      <c r="X17" s="160"/>
-      <c r="Y17" s="160"/>
+      <c r="W17" s="159"/>
+      <c r="X17" s="159"/>
+      <c r="Y17" s="159"/>
     </row>
     <row r="18" spans="2:25">
       <c r="B18" s="26" t="s">

</xml_diff>